<commit_message>
Implement batch continuation feature for previous allocations and enhance UI for file uploads
</commit_message>
<xml_diff>
--- a/sample_registration_199.xlsx
+++ b/sample_registration_199.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lerwin Loh\Desktop\Splash 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1115D04-11A7-4F27-AEFF-C418B6030977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BC67749-873C-4A2E-8343-1B92F982C6D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5364" yWindow="1908" windowWidth="15360" windowHeight="8940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Registrations_200" sheetId="1" r:id="rId1"/>
+    <sheet name="Registrations_199" sheetId="1" r:id="rId1"/>
     <sheet name="Alternate Headers" sheetId="2" r:id="rId2"/>
     <sheet name="Includes Blank Row" sheetId="3" r:id="rId3"/>
     <sheet name="Empty Template" sheetId="4" r:id="rId4"/>

</xml_diff>